<commit_message>
Actualización completa del sistema con mejoras en exportación y alertas
</commit_message>
<xml_diff>
--- a/inventario_50_registros.xlsx
+++ b/inventario_50_registros.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johanygm\Documents\vc-admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563FA8F7-0A2E-4CFC-80AE-EFCD5314DE4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CC8662-E751-423E-88A8-B24E0301CAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="173">
   <si>
     <t>codigo</t>
   </si>
@@ -539,12 +539,6 @@
   </si>
   <si>
     <t>Plateado</t>
-  </si>
-  <si>
-    <t>ACC-BC-WALLETL</t>
-  </si>
-  <si>
-    <t>ACC-GN-9FIFTY-1</t>
   </si>
 </sst>
 </file>
@@ -888,6 +882,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1821,7 +1819,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>114</v>
       </c>
@@ -1850,7 +1848,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>117</v>
       </c>
@@ -1879,7 +1877,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>120</v>
       </c>
@@ -1908,7 +1906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>123</v>
       </c>
@@ -1937,7 +1935,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>126</v>
       </c>
@@ -1966,7 +1964,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>129</v>
       </c>
@@ -1995,7 +1993,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>132</v>
       </c>
@@ -2024,7 +2022,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>135</v>
       </c>
@@ -2053,7 +2051,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>138</v>
       </c>
@@ -2082,7 +2080,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>141</v>
       </c>
@@ -2111,7 +2109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>147</v>
       </c>
@@ -2140,7 +2138,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>151</v>
       </c>
@@ -2169,10 +2167,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>174</v>
-      </c>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>154</v>
       </c>
@@ -2201,7 +2196,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>156</v>
       </c>
@@ -2230,10 +2225,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>173</v>
-      </c>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>159</v>
       </c>
@@ -2262,7 +2254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>161</v>
       </c>

</xml_diff>